<commit_message>
Make imported OT duration explicit and route moved shifts to managers
</commit_message>
<xml_diff>
--- a/public/templates/attendance-v5.xlsx
+++ b/public/templates/attendance-v5.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R51ec763772cc4ef4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Entry" sheetId="2" r:id="Re553bd0cb73641c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Examples — Do Not Upload" sheetId="3" r:id="Rc23df13d00e24a4b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Guide" sheetId="4" r:id="R2f8f5a1826024bca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R0545303613b44126"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Entry" sheetId="2" r:id="R1771a9c7c9754861"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Examples — Do Not Upload" sheetId="3" r:id="R827df3bba99d475b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Guide" sheetId="4" r:id="R87a8bf4944e44952"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -682,7 +682,7 @@
         <x:v>Values only</x:v>
       </x:c>
       <x:c r="B10" s="2" t="str">
-        <x:v>No formulas. Paste values. Payroll derives hours, lateness and authorized overtime; do not supply calculated amounts.</x:v>
+        <x:v>No formulas. Paste values. Enter requested extra-work OT hours and reason only if applying; the manager approves a quantity separately. OT start/end are optional as a pair. A late clock-out never creates OT.</x:v>
       </x:c>
       <x:c r="C10" s="1"/>
       <x:c r="D10" s="1"/>
@@ -5110,17 +5110,13 @@
         <x:v>Overtime</x:v>
       </x:c>
       <x:c r="M4" s="5" t="str">
-        <x:v>Check approved request and duration</x:v>
+        <x:v>Request one extra hour; manager decides separately</x:v>
       </x:c>
       <x:c r="N4" s="17" t="str">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="O4" s="15" t="n">
-        <x:v>46263.25</x:v>
-      </x:c>
-      <x:c r="P4" s="15" t="n">
-        <x:v>46263.291666666664</x:v>
-      </x:c>
+      <x:c r="O4" s="15" t="str"/>
+      <x:c r="P4" s="15" t="str"/>
       <x:c r="Q4" s="5" t="str">
         <x:v>Requested extra coverage; separate manager approval</x:v>
       </x:c>
@@ -8913,10 +8909,10 @@
         <x:v>Requested OT hours (optional)</x:v>
       </x:c>
       <x:c r="B15" s="2" t="str">
-        <x:v>Optional OT request (complete all OT fields)</x:v>
+        <x:v>If requesting OT: both required</x:v>
       </x:c>
       <x:c r="C15" s="2" t="str">
-        <x:v>Requested paid OT hours, not total shift hours. Requires OT start/end and a reason; manager decides the authorized hours.</x:v>
+        <x:v>Extra-work hours requested for separate manager approval, not total shift hours or a calculation from clock-out. Add a reason. OT start/end are optional as a pair; manager can approve fewer hours. Blank means no OT requested.</x:v>
       </x:c>
       <x:c r="D15" s="1"/>
       <x:c r="E15" s="1"/>
@@ -8952,10 +8948,10 @@
         <x:v>OT start date/time (optional)</x:v>
       </x:c>
       <x:c r="B16" s="2" t="str">
-        <x:v>Optional OT request (complete all OT fields)</x:v>
+        <x:v>Optional OT interval (both or neither)</x:v>
       </x:c>
       <x:c r="C16" s="2" t="str">
-        <x:v>Actual requested OT interval start, including date. Never copy a full shift as overtime.</x:v>
+        <x:v>Optional actual OT interval start, including date. Enter both OT times or neither; never copy the full shift as overtime.</x:v>
       </x:c>
       <x:c r="D16" s="1"/>
       <x:c r="E16" s="1"/>
@@ -8991,10 +8987,10 @@
         <x:v>OT end date/time (optional)</x:v>
       </x:c>
       <x:c r="B17" s="2" t="str">
-        <x:v>Optional OT request (complete all OT fields)</x:v>
+        <x:v>Optional OT interval (both or neither)</x:v>
       </x:c>
       <x:c r="C17" s="2" t="str">
-        <x:v>Requested OT interval end, including next-day date if applicable.</x:v>
+        <x:v>Optional OT interval end, including next-day date if applicable. Leave both times blank when only requested extra-work hours are known.</x:v>
       </x:c>
       <x:c r="D17" s="1"/>
       <x:c r="E17" s="1"/>
@@ -9030,7 +9026,7 @@
         <x:v>OT reason (optional)</x:v>
       </x:c>
       <x:c r="B18" s="2" t="str">
-        <x:v>Optional OT request (complete all OT fields)</x:v>
+        <x:v>If requesting OT: both required</x:v>
       </x:c>
       <x:c r="C18" s="2" t="str">
         <x:v>Why overtime was needed. Creates or links a separate approval request; attendance approval never grants OT pay.</x:v>

</xml_diff>

<commit_message>
Make imported OT duration explicit and route moved shifts to managers (#240)
</commit_message>
<xml_diff>
--- a/public/templates/attendance-v5.xlsx
+++ b/public/templates/attendance-v5.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R51ec763772cc4ef4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Entry" sheetId="2" r:id="Re553bd0cb73641c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Examples — Do Not Upload" sheetId="3" r:id="Rc23df13d00e24a4b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Guide" sheetId="4" r:id="R2f8f5a1826024bca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R0545303613b44126"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Entry" sheetId="2" r:id="R1771a9c7c9754861"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Examples — Do Not Upload" sheetId="3" r:id="R827df3bba99d475b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Guide" sheetId="4" r:id="R87a8bf4944e44952"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -682,7 +682,7 @@
         <x:v>Values only</x:v>
       </x:c>
       <x:c r="B10" s="2" t="str">
-        <x:v>No formulas. Paste values. Payroll derives hours, lateness and authorized overtime; do not supply calculated amounts.</x:v>
+        <x:v>No formulas. Paste values. Enter requested extra-work OT hours and reason only if applying; the manager approves a quantity separately. OT start/end are optional as a pair. A late clock-out never creates OT.</x:v>
       </x:c>
       <x:c r="C10" s="1"/>
       <x:c r="D10" s="1"/>
@@ -5110,17 +5110,13 @@
         <x:v>Overtime</x:v>
       </x:c>
       <x:c r="M4" s="5" t="str">
-        <x:v>Check approved request and duration</x:v>
+        <x:v>Request one extra hour; manager decides separately</x:v>
       </x:c>
       <x:c r="N4" s="17" t="str">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="O4" s="15" t="n">
-        <x:v>46263.25</x:v>
-      </x:c>
-      <x:c r="P4" s="15" t="n">
-        <x:v>46263.291666666664</x:v>
-      </x:c>
+      <x:c r="O4" s="15" t="str"/>
+      <x:c r="P4" s="15" t="str"/>
       <x:c r="Q4" s="5" t="str">
         <x:v>Requested extra coverage; separate manager approval</x:v>
       </x:c>
@@ -8913,10 +8909,10 @@
         <x:v>Requested OT hours (optional)</x:v>
       </x:c>
       <x:c r="B15" s="2" t="str">
-        <x:v>Optional OT request (complete all OT fields)</x:v>
+        <x:v>If requesting OT: both required</x:v>
       </x:c>
       <x:c r="C15" s="2" t="str">
-        <x:v>Requested paid OT hours, not total shift hours. Requires OT start/end and a reason; manager decides the authorized hours.</x:v>
+        <x:v>Extra-work hours requested for separate manager approval, not total shift hours or a calculation from clock-out. Add a reason. OT start/end are optional as a pair; manager can approve fewer hours. Blank means no OT requested.</x:v>
       </x:c>
       <x:c r="D15" s="1"/>
       <x:c r="E15" s="1"/>
@@ -8952,10 +8948,10 @@
         <x:v>OT start date/time (optional)</x:v>
       </x:c>
       <x:c r="B16" s="2" t="str">
-        <x:v>Optional OT request (complete all OT fields)</x:v>
+        <x:v>Optional OT interval (both or neither)</x:v>
       </x:c>
       <x:c r="C16" s="2" t="str">
-        <x:v>Actual requested OT interval start, including date. Never copy a full shift as overtime.</x:v>
+        <x:v>Optional actual OT interval start, including date. Enter both OT times or neither; never copy the full shift as overtime.</x:v>
       </x:c>
       <x:c r="D16" s="1"/>
       <x:c r="E16" s="1"/>
@@ -8991,10 +8987,10 @@
         <x:v>OT end date/time (optional)</x:v>
       </x:c>
       <x:c r="B17" s="2" t="str">
-        <x:v>Optional OT request (complete all OT fields)</x:v>
+        <x:v>Optional OT interval (both or neither)</x:v>
       </x:c>
       <x:c r="C17" s="2" t="str">
-        <x:v>Requested OT interval end, including next-day date if applicable.</x:v>
+        <x:v>Optional OT interval end, including next-day date if applicable. Leave both times blank when only requested extra-work hours are known.</x:v>
       </x:c>
       <x:c r="D17" s="1"/>
       <x:c r="E17" s="1"/>
@@ -9030,7 +9026,7 @@
         <x:v>OT reason (optional)</x:v>
       </x:c>
       <x:c r="B18" s="2" t="str">
-        <x:v>Optional OT request (complete all OT fields)</x:v>
+        <x:v>If requesting OT: both required</x:v>
       </x:c>
       <x:c r="C18" s="2" t="str">
         <x:v>Why overtime was needed. Creates or links a separate approval request; attendance approval never grants OT pay.</x:v>

</xml_diff>